<commit_message>
feat(auth): integrate recovery email password reset flow into dev with V19 migration
</commit_message>
<xml_diff>
--- a/frontend/test-fixtures/case1_all_valid.xlsx
+++ b/frontend/test-fixtures/case1_all_valid.xlsx
@@ -29,7 +29,7 @@
     <t>Nguyễn Văn Hợp Lệ 1</t>
   </si>
   <si>
-    <t>nv_valid1_1791232548812@company.local</t>
+    <t>nv_valid1_1791313638710@company.local</t>
   </si>
   <si>
     <t>Kỹ thuật</t>
@@ -41,7 +41,7 @@
     <t>Trần Thị Hợp Lệ 2</t>
   </si>
   <si>
-    <t>nv_valid2_1791232548812@company.local</t>
+    <t>nv_valid2_1791313638710@company.local</t>
   </si>
   <si>
     <t>Nhân sự</t>
@@ -53,7 +53,7 @@
     <t>Lê Văn Hợp Lệ 3</t>
   </si>
   <si>
-    <t>nv_valid3_1791232548812@company.local</t>
+    <t>nv_valid3_1791313638710@company.local</t>
   </si>
   <si>
     <t>Kinh doanh</t>

</xml_diff>

<commit_message>
fix(s2-01): align excel validation and improve import result UI
</commit_message>
<xml_diff>
--- a/frontend/test-fixtures/case1_all_valid.xlsx
+++ b/frontend/test-fixtures/case1_all_valid.xlsx
@@ -29,7 +29,7 @@
     <t>Nguyễn Văn Hợp Lệ 1</t>
   </si>
   <si>
-    <t>nv_valid1_1791313638710@company.local</t>
+    <t>nv_valid1_1791364218252@company.local</t>
   </si>
   <si>
     <t>Kỹ thuật</t>
@@ -41,7 +41,7 @@
     <t>Trần Thị Hợp Lệ 2</t>
   </si>
   <si>
-    <t>nv_valid2_1791313638710@company.local</t>
+    <t>nv_valid2_1791364218252@company.local</t>
   </si>
   <si>
     <t>Nhân sự</t>
@@ -53,7 +53,7 @@
     <t>Lê Văn Hợp Lệ 3</t>
   </si>
   <si>
-    <t>nv_valid3_1791313638710@company.local</t>
+    <t>nv_valid3_1791364218252@company.local</t>
   </si>
   <si>
     <t>Kinh doanh</t>

</xml_diff>

<commit_message>
feat(org-chart): fix organizational chart tree layout, connectors and employee count
</commit_message>
<xml_diff>
--- a/frontend/test-fixtures/case1_all_valid.xlsx
+++ b/frontend/test-fixtures/case1_all_valid.xlsx
@@ -29,7 +29,7 @@
     <t>Nguyễn Văn Hợp Lệ 1</t>
   </si>
   <si>
-    <t>nv_valid1_1791364218252@company.local</t>
+    <t>nv_valid1_1791476314118@company.local</t>
   </si>
   <si>
     <t>Kỹ thuật</t>
@@ -41,7 +41,7 @@
     <t>Trần Thị Hợp Lệ 2</t>
   </si>
   <si>
-    <t>nv_valid2_1791364218252@company.local</t>
+    <t>nv_valid2_1791476314118@company.local</t>
   </si>
   <si>
     <t>Nhân sự</t>
@@ -53,7 +53,7 @@
     <t>Lê Văn Hợp Lệ 3</t>
   </si>
   <si>
-    <t>nv_valid3_1791364218252@company.local</t>
+    <t>nv_valid3_1791476314118@company.local</t>
   </si>
   <si>
     <t>Kinh doanh</t>

</xml_diff>

<commit_message>
fix(sprint2): align S2-10 requisition scoping, draft validation, test compatibility and Excel fixtures
</commit_message>
<xml_diff>
--- a/frontend/test-fixtures/case1_all_valid.xlsx
+++ b/frontend/test-fixtures/case1_all_valid.xlsx
@@ -29,7 +29,7 @@
     <t>Nguyễn Văn Hợp Lệ 1</t>
   </si>
   <si>
-    <t>nv_valid1_1791476314118@company.local</t>
+    <t>nv_valid1_1791567428307@company.local</t>
   </si>
   <si>
     <t>Kỹ thuật</t>
@@ -41,7 +41,7 @@
     <t>Trần Thị Hợp Lệ 2</t>
   </si>
   <si>
-    <t>nv_valid2_1791476314118@company.local</t>
+    <t>nv_valid2_1791567428307@company.local</t>
   </si>
   <si>
     <t>Nhân sự</t>
@@ -53,7 +53,7 @@
     <t>Lê Văn Hợp Lệ 3</t>
   </si>
   <si>
-    <t>nv_valid3_1791476314118@company.local</t>
+    <t>nv_valid3_1791567428307@company.local</t>
   </si>
   <si>
     <t>Kinh doanh</t>

</xml_diff>

<commit_message>
chore: update excel test fixtures from test run
</commit_message>
<xml_diff>
--- a/frontend/test-fixtures/case1_all_valid.xlsx
+++ b/frontend/test-fixtures/case1_all_valid.xlsx
@@ -29,7 +29,7 @@
     <t>Nguyễn Văn Hợp Lệ 1</t>
   </si>
   <si>
-    <t>nv_valid1_1791567428307@company.local</t>
+    <t>nv_valid1_1791567643572@company.local</t>
   </si>
   <si>
     <t>Kỹ thuật</t>
@@ -41,7 +41,7 @@
     <t>Trần Thị Hợp Lệ 2</t>
   </si>
   <si>
-    <t>nv_valid2_1791567428307@company.local</t>
+    <t>nv_valid2_1791567643572@company.local</t>
   </si>
   <si>
     <t>Nhân sự</t>
@@ -53,7 +53,7 @@
     <t>Lê Văn Hợp Lệ 3</t>
   </si>
   <si>
-    <t>nv_valid3_1791567428307@company.local</t>
+    <t>nv_valid3_1791567643572@company.local</t>
   </si>
   <si>
     <t>Kinh doanh</t>

</xml_diff>

<commit_message>
feat(system): standardize pagination across modules, enforce unique phone number constraints, and refine UI components
</commit_message>
<xml_diff>
--- a/frontend/test-fixtures/case1_all_valid.xlsx
+++ b/frontend/test-fixtures/case1_all_valid.xlsx
@@ -29,7 +29,7 @@
     <t>Nguyễn Văn Hợp Lệ 1</t>
   </si>
   <si>
-    <t>nv_valid1_1791567643572@company.local</t>
+    <t>nv_valid1_1791909724777@company.local</t>
   </si>
   <si>
     <t>Kỹ thuật</t>
@@ -41,7 +41,7 @@
     <t>Trần Thị Hợp Lệ 2</t>
   </si>
   <si>
-    <t>nv_valid2_1791567643572@company.local</t>
+    <t>nv_valid2_1791909724777@company.local</t>
   </si>
   <si>
     <t>Nhân sự</t>
@@ -53,7 +53,7 @@
     <t>Lê Văn Hợp Lệ 3</t>
   </si>
   <si>
-    <t>nv_valid3_1791567643572@company.local</t>
+    <t>nv_valid3_1791909724777@company.local</t>
   </si>
   <si>
     <t>Kinh doanh</t>

</xml_diff>

<commit_message>
feat(recruitment-e2e): integrate recruitment lifecycle, persistent CV upload, and PostgreSQL V32 migration
</commit_message>
<xml_diff>
--- a/frontend/test-fixtures/case1_all_valid.xlsx
+++ b/frontend/test-fixtures/case1_all_valid.xlsx
@@ -29,7 +29,7 @@
     <t>Nguyễn Văn Hợp Lệ 1</t>
   </si>
   <si>
-    <t>nv_valid1_1791567643572@company.local</t>
+    <t>nv_valid1_1792700857270@company.local</t>
   </si>
   <si>
     <t>Kỹ thuật</t>
@@ -41,7 +41,7 @@
     <t>Trần Thị Hợp Lệ 2</t>
   </si>
   <si>
-    <t>nv_valid2_1791567643572@company.local</t>
+    <t>nv_valid2_1792700857270@company.local</t>
   </si>
   <si>
     <t>Nhân sự</t>
@@ -53,7 +53,7 @@
     <t>Lê Văn Hợp Lệ 3</t>
   </si>
   <si>
-    <t>nv_valid3_1791567643572@company.local</t>
+    <t>nv_valid3_1792700857270@company.local</t>
   </si>
   <si>
     <t>Kinh doanh</t>

</xml_diff>